<commit_message>
Adding usbcam/cam application for V7.00 AISDK
</commit_message>
<xml_diff>
--- a/13_Car_ahead_departure_detection/Car_ahead_departure_detection_cam/exe/tiny_yolov3_cam/tiny_yolov3_cam_summary.xlsx
+++ b/13_Car_ahead_departure_detection/Car_ahead_departure_detection_cam/exe/tiny_yolov3_cam/tiny_yolov3_cam_summary.xlsx
@@ -892,7 +892,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>input.4</t>
+          <t>146</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -952,7 +952,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>input.8</t>
+          <t>78</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1012,7 +1012,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>input.16</t>
+          <t>149</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1072,7 +1072,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>input.20</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1132,7 +1132,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>input.28</t>
+          <t>152</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1192,7 +1192,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>input.32</t>
+          <t>86</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1252,7 +1252,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>input.40</t>
+          <t>155</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>input.44</t>
+          <t>90</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>input.52</t>
+          <t>158</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1432,7 +1432,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>input.56</t>
+          <t>94</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1492,7 +1492,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>input.64</t>
+          <t>161</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>input.68</t>
+          <t>121</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1612,7 +1612,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>input.76</t>
+          <t>164</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>input.88</t>
+          <t>167</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>input.100</t>
+          <t>170</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1852,7 +1852,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>input.116</t>
+          <t>173</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1912,7 +1912,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>onnx::Concat_140</t>
+          <t>140</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1972,7 +1972,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>input.132</t>
+          <t>176</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">

</xml_diff>